<commit_message>
Small fixes on env units
</commit_message>
<xml_diff>
--- a/results/technical_validation/summary_metallican_2023_updated.xlsx
+++ b/results/technical_validation/summary_metallican_2023_updated.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,7 +513,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Cobalt</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,17 +523,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>142285</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Concentrate</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>216587.250461</v>
+        <v>142285</v>
       </c>
     </row>
     <row r="7">
@@ -558,16 +558,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Matte</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>278281.1182</v>
+        <v>13720</v>
       </c>
     </row>
     <row r="8">
@@ -578,62 +578,62 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate and doré produced</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>12154</v>
+        <v>57900</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Diamonds</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Concentrate</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4200000.337542</v>
+        <v>189187.250461</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Diamonds</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4600000</v>
+        <v>233023.1182</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Diamonds</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -643,11 +643,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Carats recovered</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.02</v>
+        <v>12154</v>
       </c>
     </row>
     <row r="12">
@@ -658,116 +658,116 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Diamond recovered</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.6679524060000001</v>
+        <v>4200000.337542</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ferroniobium</t>
+          <t>Diamonds</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11700</v>
+        <v>4600000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GEOs</t>
+          <t>Diamonds</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Carats recovered</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0003172557</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Diamonds</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ore delivered</t>
+          <t>Diamond recovered</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>33245</v>
+        <v>0.6679524060000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Ferroniobium</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ore milled</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1374194</v>
+        <v>11700</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>GEOs</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Intermediate metal</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>43090380.5081444</v>
+        <v>0.0003172557</v>
       </c>
     </row>
     <row r="18">
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Ore delivered</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>16333305</v>
+        <v>33245</v>
       </c>
     </row>
     <row r="19">
@@ -798,16 +798,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Ore milled</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>164.8935094431374</v>
+        <v>1374194</v>
       </c>
     </row>
     <row r="20">
@@ -818,16 +818,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contained metal in concentrate </t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4.3869931575</v>
+        <v>43090380.5081444</v>
       </c>
     </row>
     <row r="21">
@@ -838,16 +838,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate and doré produced</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5.8276450705</v>
+        <v>16567976</v>
       </c>
     </row>
     <row r="22">
@@ -863,11 +863,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2.6938803557</v>
+        <v>161.9005129486374</v>
       </c>
     </row>
     <row r="23">
@@ -883,57 +883,57 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Metal in doré produced</t>
+          <t xml:space="preserve">Contained metal in concentrate </t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.2515737365</v>
+        <v>4.3869931575</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>21000000</v>
+        <v>5.8276450705</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Intermediate metal</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>43740000</v>
+        <v>2.6938803557</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -943,11 +943,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Metal in doré produced</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>28013117.54684838</v>
+        <v>1.2515737365</v>
       </c>
     </row>
     <row r="27">
@@ -958,16 +958,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Concentrate &amp; pellets</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>22400000</v>
+        <v>26600000</v>
       </c>
     </row>
     <row r="28">
@@ -978,7 +978,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -998,36 +998,36 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24200000</v>
+        <v>60239000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Refinery production</t>
+          <t>Concentrate</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>244600</v>
+        <v>21813117.54684838</v>
       </c>
     </row>
     <row r="31">
@@ -1038,36 +1038,36 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1225</v>
+        <v>244600</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>407034</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="33">
@@ -1078,22 +1078,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33120</v>
+        <v>407034</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Molybdenum</t>
+          <t>Lithium</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1103,31 +1103,31 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Concentrate</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1445.217584</v>
+        <v>33120</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Nickel</t>
+          <t>Molybdenum</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>9220</v>
+        <v>1445.217584</v>
       </c>
     </row>
     <row r="36">
@@ -1138,16 +1138,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Refinery production</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>32268</v>
+        <v>1082352.941176471</v>
       </c>
     </row>
     <row r="37">
@@ -1158,16 +1158,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Matte</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>200</v>
+        <v>62251</v>
       </c>
     </row>
     <row r="38">
@@ -1178,56 +1178,56 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>59600</v>
+        <v>70468</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Nickel, cobalt</t>
+          <t>Nickel</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Refinery production</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>35636</v>
+        <v>62382</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>Niobium</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mill feed</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1488757</v>
+        <v>2200000</v>
       </c>
     </row>
     <row r="41">
@@ -1243,11 +1243,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ore milled</t>
+          <t>Mill feed</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>55654870</v>
+        <v>1488757</v>
       </c>
     </row>
     <row r="42">
@@ -1263,11 +1263,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Ore milled</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>62264839.289214</v>
+        <v>55654870</v>
       </c>
     </row>
     <row r="43">
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Material mined</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1855271</v>
+        <v>86423235.61795826</v>
       </c>
     </row>
     <row r="44">
@@ -1303,11 +1303,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Material mined</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>140449778</v>
+        <v>1855271</v>
       </c>
     </row>
     <row r="45">
@@ -1323,37 +1323,37 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tonnes mined</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>50015000</v>
+        <v>141322971</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PGM</t>
+          <t>Ore</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Tonnes mined</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>38.319512</v>
+        <v>50015000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>PGM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.2504042449</v>
+        <v>38.319512</v>
       </c>
     </row>
     <row r="48">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Metal in doré produced</t>
+          <t>Intermediate metal</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3.036634705</v>
+        <v>1.2504042449</v>
       </c>
     </row>
     <row r="49">
@@ -1398,16 +1398,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Metal in doré produced</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>155.018351032</v>
+        <v>3.036634705</v>
       </c>
     </row>
     <row r="50">
@@ -1423,31 +1423,31 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate and doré produced</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>26.4915663305</v>
+        <v>155.018351032</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EAF production</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>828000</v>
+        <v>26.4915663305</v>
       </c>
     </row>
     <row r="52">
@@ -1458,16 +1458,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Flat</t>
+          <t>EAF production</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>3100000</v>
+        <v>828000</v>
       </c>
     </row>
     <row r="53">
@@ -1483,17 +1483,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Long/wire rod, bars, slabs</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1900000</v>
+        <v>3100000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Titanium dioxide slag</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1503,57 +1503,57 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Long/wire rod, bars, slabs</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1111000</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Uranium</t>
+          <t>Titanium dioxide slag</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>21137.3872</v>
+        <v>1111000</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Zinc</t>
+          <t>Uranium</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Refinery production</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1008600</v>
+        <v>142135.7272203253</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Zinc</t>
+          <t>Uranium</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1563,11 +1563,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>108040.997133</v>
+        <v>21137.3872</v>
       </c>
     </row>
     <row r="58">
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>74581</v>
+        <v>1008600</v>
       </c>
     </row>
     <row r="59">
@@ -1603,10 +1603,50 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
+          <t>Concentrate</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>69440.997133</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Zinc</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Usable ore</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Contained metal in concentrate</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>74581</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Zinc</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Usable ore</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
           <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D61" t="n">
         <v>34642</v>
       </c>
     </row>

</xml_diff>

<commit_message>
More transparent source ids and
</commit_message>
<xml_diff>
--- a/results/technical_validation/summary_metallican_2023_updated.xlsx
+++ b/results/technical_validation/summary_metallican_2023_updated.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,11 +603,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>189187.250461</v>
+        <v>337008.012277</v>
       </c>
     </row>
     <row r="10">
@@ -623,31 +623,31 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>233023.1182</v>
+        <v>12154</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Diamonds</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate and doré produced</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>12154</v>
+        <v>4200000.337542</v>
       </c>
     </row>
     <row r="12">
@@ -658,16 +658,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4200000.337542</v>
+        <v>4600000</v>
       </c>
     </row>
     <row r="13">
@@ -678,16 +678,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Carats recovered</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4600000</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="14">
@@ -703,71 +703,71 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Carats recovered</t>
+          <t>Diamond recovered</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.02</v>
+        <v>0.6679524060000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Diamonds</t>
+          <t>Ferroniobium</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Diamond recovered</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.6679524060000001</v>
+        <v>11700</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ferroniobium</t>
+          <t>GEOs</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Contained metal in doré</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11700</v>
+        <v>0.0003172557</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GEOs</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Ore delivered</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0003172557</v>
+        <v>33245</v>
       </c>
     </row>
     <row r="18">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ore delivered</t>
+          <t>Ore milled</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>33245</v>
+        <v>1374194</v>
       </c>
     </row>
     <row r="19">
@@ -803,11 +803,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ore milled</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1374194</v>
+        <v>43090380.5081444</v>
       </c>
     </row>
     <row r="20">
@@ -818,16 +818,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>43090380.5081444</v>
+        <v>16567976</v>
       </c>
     </row>
     <row r="21">
@@ -838,16 +838,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16567976</v>
+        <v>5.8276450705</v>
       </c>
     </row>
     <row r="22">
@@ -863,77 +863,77 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Contained metal in doré</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>161.9005129486374</v>
+        <v>162.115404403198</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contained metal in concentrate </t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.3869931575</v>
+        <v>5600000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate and doré produced</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5.8276450705</v>
+        <v>53625000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2.6938803557</v>
+        <v>244600</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -943,177 +943,177 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metal in doré produced</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.2515737365</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Lithium</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>26600000</v>
+        <v>407034</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Lithium</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Iron ore</t>
+          <t>Concentrate</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>5901000</v>
+        <v>33120</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Molybdenum</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>60239000</v>
+        <v>1445.217584</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Nickel</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>21813117.54684838</v>
+        <v>1082352.941176471</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Nickel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Refinery production</t>
+          <t>Matte</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>244600</v>
+        <v>62251</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Nickel</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1225</v>
+        <v>70468</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>Nickel</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>407034</v>
+        <v>111262</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>Niobium</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Concentrate</t>
+          <t>Ore mined</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>33120</v>
+        <v>2200000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Molybdenum</t>
+          <t>Niobium</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1127,13 +1127,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1445.217584</v>
+        <v>6568.95</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Nickel</t>
+          <t>Ore</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1143,77 +1143,77 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Mill feed</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1082352.941176471</v>
+        <v>1488757</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Nickel</t>
+          <t>Ore</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Matte</t>
+          <t>Ore milled</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>62251</v>
+        <v>55654870</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Nickel</t>
+          <t>Ore</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Refinery production</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>70468</v>
+        <v>86438311.65746826</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Nickel</t>
+          <t>Ore</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Total extraction</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate</t>
+          <t>Material mined</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>62382</v>
+        <v>1855271</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Niobium</t>
+          <t>Ore</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1227,193 +1227,193 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2200000</v>
+        <v>141322971</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>PGM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mill feed</t>
+          <t>Contained metal in doré</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1488757</v>
+        <v>38.319512</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>PGMs</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ore milled</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>55654870</v>
+        <v>4.41607493</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Crude ore</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ore processed</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>86423235.61795826</v>
+        <v>26.4915663305</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Material mined</t>
+          <t>Contained metal in doré</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1855271</v>
+        <v>136.3090172569</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Intermediate metal produced</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ore mined</t>
+          <t>EAF production</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>141322971</v>
+        <v>828000</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ore</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Total extraction</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tonnes mined</t>
+          <t>Flat</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>50015000</v>
+        <v>3100000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PGM</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Long/wire rod, bars, slabs</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>38.319512</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Titanium dioxide slag</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Intermediate metal</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1.2504042449</v>
+        <v>1111000</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Uranium</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Crude ore</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Metal in doré produced</t>
+          <t>Ore processed</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>3.036634705</v>
+        <v>142135.7272203253</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Uranium</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1427,226 +1427,66 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>155.018351032</v>
+        <v>21137.3872</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Zinc</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Usable ore</t>
+          <t>Refined metal produced</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Contained metal in concentrate and doré produced</t>
+          <t>Refinery production</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>26.4915663305</v>
+        <v>1008600</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Zinc</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Intermediate metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>EAF production</t>
+          <t>Contained metal in concentrate</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>828000</v>
+        <v>47641.438517</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Zinc</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Refined metal produced</t>
+          <t>Usable ore</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Flat</t>
+          <t>Contained metal in concentrate and doré produced</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3100000</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Steel</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Refined metal produced</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Long/wire rod, bars, slabs</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>1900000</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Titanium dioxide slag</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Refined metal produced</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>1111000</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Uranium</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Crude ore</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Ore processed</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>142135.7272203253</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Uranium</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Usable ore</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Contained metal in concentrate</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>21137.3872</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Zinc</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Refined metal produced</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Refinery production</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>1008600</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Zinc</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Usable ore</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Concentrate</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>69440.997133</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Zinc</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Usable ore</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Contained metal in concentrate</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>74581</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Zinc</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Usable ore</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Contained metal in concentrate and doré produced</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
         <v>34642</v>
       </c>
     </row>

</xml_diff>